<commit_message>
add full reports system
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,81 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fee</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>visit_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>زهرا</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9144415789</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>حجامت</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>600000</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>مینا</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>04433665565</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>زالو</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2 عدد زالو از پاها</t>
         </is>
       </c>
     </row>

</xml_diff>